<commit_message>
Subindo Update do md csv e pdf
</commit_message>
<xml_diff>
--- a/documents/datasets/exemplos-us-por-dominio.xlsx
+++ b/documents/datasets/exemplos-us-por-dominio.xlsx
@@ -62,19 +62,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:J26"/>
+  <dimension ref="A1:L26"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
     <col min="3" max="3" width="26" customWidth="1"/>
-    <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="4" max="4" width="55" customWidth="1"/>
     <col min="5" max="5" width="12" customWidth="1"/>
-    <col min="6" max="6" width="10" customWidth="1"/>
-    <col min="7" max="7" width="40" customWidth="1"/>
-    <col min="8" max="8" width="16" customWidth="1"/>
-    <col min="9" max="9" width="26" customWidth="1"/>
-    <col min="10" max="10" width="90" customWidth="1"/>
+    <col min="6" max="6" width="14" customWidth="1"/>
+    <col min="7" max="7" width="12" customWidth="1"/>
+    <col min="8" max="8" width="9" customWidth="1"/>
+    <col min="9" max="9" width="40" customWidth="1"/>
+    <col min="10" max="10" width="16" customWidth="1"/>
+    <col min="11" max="11" width="26" customWidth="1"/>
+    <col min="12" max="12" width="85" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -95,35 +97,45 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">equivalent_ml_task_labels</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">num_ml_task_labels</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">domain_confidence</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">id</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">abstract</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">abstract_theme</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">llm</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">role_shorten</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">user_story</t>
         </is>
@@ -145,35 +157,43 @@
       </c>
       <c r="D2" s="0" t="inlineStr">
         <is>
+          <t xml:space="preserve">Ranking; Matching; Pricing; Advertising; Entity Resolution; Sentiment Analysis; Bias Detection in Language Models</t>
+        </is>
+      </c>
+      <c r="E2" s="0">
+        <v>7</v>
+      </c>
+      <c r="F2" s="0" t="inlineStr">
+        <is>
           <t xml:space="preserve">Medium</t>
         </is>
       </c>
-      <c r="E2" s="0" t="inlineStr">
+      <c r="G2" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A23US9O1</t>
         </is>
       </c>
-      <c r="F2" s="0" t="inlineStr">
+      <c r="H2" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A23</t>
         </is>
       </c>
-      <c r="G2" s="0" t="inlineStr">
+      <c r="I2" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Search-engine bias analysis (PAWS platform)</t>
         </is>
       </c>
-      <c r="H2" s="0" t="inlineStr">
+      <c r="J2" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">O1_mini</t>
         </is>
       </c>
-      <c r="I2" s="0" t="inlineStr">
+      <c r="K2" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">competitor in the search engine market</t>
         </is>
       </c>
-      <c r="J2" s="0" t="inlineStr">
+      <c r="L2" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">As a competitor in the search engine market, I want to analyze how our ranking algorithms compare to others using PAWS, so that I can identify areas for improvement and differentiation.</t>
         </is>
@@ -195,35 +215,43 @@
       </c>
       <c r="D3" s="0" t="inlineStr">
         <is>
+          <t xml:space="preserve">Classification; Representation Learning; Clustering; Anomaly Detection; Subset Selection</t>
+        </is>
+      </c>
+      <c r="E3" s="0">
+        <v>5</v>
+      </c>
+      <c r="F3" s="0" t="inlineStr">
+        <is>
           <t xml:space="preserve">Medium</t>
         </is>
       </c>
-      <c r="E3" s="0" t="inlineStr">
+      <c r="G3" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A2US3Ge</t>
         </is>
       </c>
-      <c r="F3" s="0" t="inlineStr">
+      <c r="H3" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A2</t>
         </is>
       </c>
-      <c r="G3" s="0" t="inlineStr">
+      <c r="I3" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Wearable-based detection of physical aggression in children</t>
         </is>
       </c>
-      <c r="H3" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Gemini_1.5_flash</t>
-        </is>
-      </c>
-      <c r="I3" s="0" t="inlineStr">
+      <c r="J3" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gemini_1.5_flash</t>
+        </is>
+      </c>
+      <c r="K3" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">therapist</t>
         </is>
       </c>
-      <c r="J3" s="0" t="inlineStr">
+      <c r="L3" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">As a therapist working with aggressive children, I want objective data on their physical activity patterns to track progress in anger management and de-escalation techniques.</t>
         </is>
@@ -245,35 +273,43 @@
       </c>
       <c r="D4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">High</t>
-        </is>
-      </c>
-      <c r="E4" s="0" t="inlineStr">
+          <t xml:space="preserve">Classification; Regression; Ranking; Representation Learning; Clustering; Anomaly Detection; Spatio-Temporal Process Learning; Graph Mining; Sentiment Analysis; Bias Detection in Word Embeddings; Bias Detection in Language Models; Machine Translation; Speech Recognition</t>
+        </is>
+      </c>
+      <c r="E4" s="0">
+        <v>13</v>
+      </c>
+      <c r="F4" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="G4" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A1US1Ge</t>
         </is>
       </c>
-      <c r="F4" s="0" t="inlineStr">
+      <c r="H4" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A1</t>
         </is>
       </c>
-      <c r="G4" s="0" t="inlineStr">
+      <c r="I4" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Autonomous vehicles (AI + real-time data for perception &amp; collision avoidance)</t>
         </is>
       </c>
-      <c r="H4" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Gemini_1.5_flash</t>
-        </is>
-      </c>
-      <c r="I4" s="0" t="inlineStr">
+      <c r="J4" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gemini_1.5_flash</t>
+        </is>
+      </c>
+      <c r="K4" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">driver</t>
         </is>
       </c>
-      <c r="J4" s="0" t="inlineStr">
+      <c r="L4" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">As a driver, I want a car that uses AI and real-time data to react faster than humans in emergency situations, reducing my risk of accidents.</t>
         </is>
@@ -295,35 +331,43 @@
       </c>
       <c r="D5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">High</t>
-        </is>
-      </c>
-      <c r="E5" s="0" t="inlineStr">
+          <t xml:space="preserve">Classification</t>
+        </is>
+      </c>
+      <c r="E5" s="0">
+        <v>1</v>
+      </c>
+      <c r="F5" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="G5" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A15US7O1</t>
         </is>
       </c>
-      <c r="F5" s="0" t="inlineStr">
+      <c r="H5" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A15</t>
         </is>
       </c>
-      <c r="G5" s="0" t="inlineStr">
+      <c r="I5" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Income / poverty prediction from demographic &amp; lifestyle data</t>
         </is>
       </c>
-      <c r="H5" s="0" t="inlineStr">
+      <c r="J5" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">O1_mini</t>
         </is>
       </c>
-      <c r="I5" s="0" t="inlineStr">
+      <c r="K5" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">non-profit organization leader</t>
         </is>
       </c>
-      <c r="J5" s="0" t="inlineStr">
+      <c r="L5" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">As a nonprofit organization leader, I want to analyze income prediction data, so that I can develop programs that effectively target and alleviate economic disparities within communities.</t>
         </is>
@@ -345,35 +389,43 @@
       </c>
       <c r="D6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">High</t>
-        </is>
-      </c>
-      <c r="E6" s="0" t="inlineStr">
+          <t xml:space="preserve">Classification</t>
+        </is>
+      </c>
+      <c r="E6" s="0">
+        <v>1</v>
+      </c>
+      <c r="F6" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="G6" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A19US1Ll</t>
         </is>
       </c>
-      <c r="F6" s="0" t="inlineStr">
+      <c r="H6" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A19</t>
         </is>
       </c>
-      <c r="G6" s="0" t="inlineStr">
+      <c r="I6" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Credit-card default prediction</t>
         </is>
       </c>
-      <c r="H6" s="0" t="inlineStr">
+      <c r="J6" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Llama 3.1 70b</t>
         </is>
       </c>
-      <c r="I6" s="0" t="inlineStr">
+      <c r="K6" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">banker</t>
         </is>
       </c>
-      <c r="J6" s="0" t="inlineStr">
+      <c r="L6" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">As a banker, I want to minimize credit risk and optimize lending decisions, so I need a reliable method to predict credit card default rates using data analytics.</t>
         </is>
@@ -395,35 +447,43 @@
       </c>
       <c r="D7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">High</t>
-        </is>
-      </c>
-      <c r="E7" s="0" t="inlineStr">
+          <t xml:space="preserve">Districting; Task Assignment; Resource Allocation</t>
+        </is>
+      </c>
+      <c r="E7" s="0">
+        <v>3</v>
+      </c>
+      <c r="F7" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="G7" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A5US2Ge</t>
         </is>
       </c>
-      <c r="F7" s="0" t="inlineStr">
+      <c r="H7" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A5</t>
         </is>
       </c>
-      <c r="G7" s="0" t="inlineStr">
+      <c r="I7" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">GoCart autonomous delivery robot in healthcare/residential facilities</t>
         </is>
       </c>
-      <c r="H7" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Gemini_1.5_flash</t>
-        </is>
-      </c>
-      <c r="I7" s="0" t="inlineStr">
+      <c r="J7" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gemini_1.5_flash</t>
+        </is>
+      </c>
+      <c r="K7" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">lab technician</t>
         </is>
       </c>
-      <c r="J7" s="0" t="inlineStr">
+      <c r="L7" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">As a lab technician, I want to easily track the location and status of blood and urine samples using the robot to ensure timely processing.</t>
         </is>
@@ -445,35 +505,43 @@
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
+          <t xml:space="preserve">Representation Learning; Anomaly Detection; Data Summarization; Entity Resolution; Bias Detection in Language Models</t>
+        </is>
+      </c>
+      <c r="E8" s="0">
+        <v>5</v>
+      </c>
+      <c r="F8" s="0" t="inlineStr">
+        <is>
           <t xml:space="preserve">Medium</t>
         </is>
       </c>
-      <c r="E8" s="0" t="inlineStr">
+      <c r="G8" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A11US2Ge</t>
         </is>
       </c>
-      <c r="F8" s="0" t="inlineStr">
+      <c r="H8" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A11</t>
         </is>
       </c>
-      <c r="G8" s="0" t="inlineStr">
+      <c r="I8" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Anti-counterfeiting copy-detection patterns (digital twin, image-to-image GANs)</t>
         </is>
       </c>
-      <c r="H8" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Gemini_1.5_flash</t>
-        </is>
-      </c>
-      <c r="I8" s="0" t="inlineStr">
+      <c r="J8" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gemini_1.5_flash</t>
+        </is>
+      </c>
+      <c r="K8" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">printing press operator</t>
         </is>
       </c>
-      <c r="J8" s="0" t="inlineStr">
+      <c r="L8" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">As a printing press operator, I want the platform to analyze digital templates containing CDPs and predict how they will appear on the final printed product, ensuring accurate replication.</t>
         </is>
@@ -495,35 +563,43 @@
       </c>
       <c r="D9" s="0" t="inlineStr">
         <is>
+          <t xml:space="preserve">Ranking</t>
+        </is>
+      </c>
+      <c r="E9" s="0">
+        <v>1</v>
+      </c>
+      <c r="F9" s="0" t="inlineStr">
+        <is>
           <t xml:space="preserve">Medium</t>
         </is>
       </c>
-      <c r="E9" s="0" t="inlineStr">
+      <c r="G9" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A28US1Ge</t>
         </is>
       </c>
-      <c r="F9" s="0" t="inlineStr">
+      <c r="H9" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A28</t>
         </is>
       </c>
-      <c r="G9" s="0" t="inlineStr">
+      <c r="I9" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Reciprocal dating recommender from speed-dating data</t>
         </is>
       </c>
-      <c r="H9" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Gemini_1.5_flash</t>
-        </is>
-      </c>
-      <c r="I9" s="0" t="inlineStr">
+      <c r="J9" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gemini_1.5_flash</t>
+        </is>
+      </c>
+      <c r="K9" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">single person</t>
         </is>
       </c>
-      <c r="J9" s="0" t="inlineStr">
+      <c r="L9" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">As a single person looking for love, I want a dating recommender system that goes beyond self- reported profiles and considers real- life interactions and compatibility.</t>
         </is>
@@ -545,35 +621,43 @@
       </c>
       <c r="D10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">High</t>
-        </is>
-      </c>
-      <c r="E10" s="0" t="inlineStr">
+          <t xml:space="preserve">Classification; Regression; Ranking; Anomaly Detection; Entity Resolution; Sentiment Analysis; Bias Detection in Word Embeddings; Bias Detection in Language Models; Machine Translation; Speech Recognition</t>
+        </is>
+      </c>
+      <c r="E10" s="0">
+        <v>10</v>
+      </c>
+      <c r="F10" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="G10" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A9US1O1</t>
         </is>
       </c>
-      <c r="F10" s="0" t="inlineStr">
+      <c r="H10" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A9</t>
         </is>
       </c>
-      <c r="G10" s="0" t="inlineStr">
+      <c r="I10" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Heart disease diagnosis with Fuzzy SVM &amp; incremental learning</t>
         </is>
       </c>
-      <c r="H10" s="0" t="inlineStr">
+      <c r="J10" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">O1_mini</t>
         </is>
       </c>
-      <c r="I10" s="0" t="inlineStr">
+      <c r="K10" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">cardiologist</t>
         </is>
       </c>
-      <c r="J10" s="0" t="inlineStr">
+      <c r="L10" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">As a cardiologist, I want the system to quickly analyze patient data using incremental Fuzzy SVM, so I can receive timely and accurate heart disease diagnoses.</t>
         </is>
@@ -595,35 +679,43 @@
       </c>
       <c r="D11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">High</t>
-        </is>
-      </c>
-      <c r="E11" s="0" t="inlineStr">
+          <t xml:space="preserve">Classification; Regression; Ranking; Representation Learning; Anomaly Detection; Spatio-Temporal Process Learning; Graph Diffusion; Graph Augmentation; Subset Selection; Data Summarization; Graph Mining; Entity Resolution; Sentiment Analysis; Bias Detection in Word Embeddings; Bias Detection in Language Models; Machine Translation; Speech Recognition</t>
+        </is>
+      </c>
+      <c r="E11" s="0">
+        <v>17</v>
+      </c>
+      <c r="F11" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="G11" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A34US1Ge</t>
         </is>
       </c>
-      <c r="F11" s="0" t="inlineStr">
+      <c r="H11" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A34</t>
         </is>
       </c>
-      <c r="G11" s="0" t="inlineStr">
+      <c r="I11" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">DNN-based network intrusion detection system</t>
         </is>
       </c>
-      <c r="H11" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Gemini_1.5_flash</t>
-        </is>
-      </c>
-      <c r="I11" s="0" t="inlineStr">
+      <c r="J11" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gemini_1.5_flash</t>
+        </is>
+      </c>
+      <c r="K11" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">analyst</t>
         </is>
       </c>
-      <c r="J11" s="0" t="inlineStr">
+      <c r="L11" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">As a cybersecurity analyst, I want to utilize a DNN- based IDS that can detect and classify new and unpredictable cyberattacks automatically, ensuring our network remains secure against evolving threats.</t>
         </is>
@@ -645,35 +737,43 @@
       </c>
       <c r="D12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">High</t>
-        </is>
-      </c>
-      <c r="E12" s="0" t="inlineStr">
+          <t xml:space="preserve">Classification</t>
+        </is>
+      </c>
+      <c r="E12" s="0">
+        <v>1</v>
+      </c>
+      <c r="F12" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="G12" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A29US1Ge</t>
         </is>
       </c>
-      <c r="F12" s="0" t="inlineStr">
+      <c r="H12" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A29</t>
         </is>
       </c>
-      <c r="G12" s="0" t="inlineStr">
+      <c r="I12" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Historical census record linkage</t>
         </is>
       </c>
-      <c r="H12" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Gemini_1.5_flash</t>
-        </is>
-      </c>
-      <c r="I12" s="0" t="inlineStr">
+      <c r="J12" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gemini_1.5_flash</t>
+        </is>
+      </c>
+      <c r="K12" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">economic historian</t>
         </is>
       </c>
-      <c r="J12" s="0" t="inlineStr">
+      <c r="L12" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">As an economic historian, I want to analyze the long- term effects of early life conditions on individuals' later life outcomes, but I need a reliable way to track individuals across historical census records.</t>
         </is>
@@ -695,35 +795,43 @@
       </c>
       <c r="D13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">High</t>
-        </is>
-      </c>
-      <c r="E13" s="0" t="inlineStr">
+          <t xml:space="preserve">Regression</t>
+        </is>
+      </c>
+      <c r="E13" s="0">
+        <v>1</v>
+      </c>
+      <c r="F13" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="G13" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A10US6Ge</t>
         </is>
       </c>
-      <c r="F13" s="0" t="inlineStr">
+      <c r="H13" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A10</t>
         </is>
       </c>
-      <c r="G13" s="0" t="inlineStr">
+      <c r="I13" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Blood-glucose / hypoglycemia prediction with Support Vector Regression</t>
         </is>
       </c>
-      <c r="H13" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Gemini_1.5_flash</t>
-        </is>
-      </c>
-      <c r="I13" s="0" t="inlineStr">
+      <c r="J13" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gemini_1.5_flash</t>
+        </is>
+      </c>
+      <c r="K13" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">health insurance provider</t>
         </is>
       </c>
-      <c r="J13" s="0" t="inlineStr">
+      <c r="L13" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">As a health insurance provider, I want to see if this model can be used to reduce the risk of complications and hospitalizations for people with diabetes.</t>
         </is>
@@ -745,35 +853,43 @@
       </c>
       <c r="D14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">High</t>
-        </is>
-      </c>
-      <c r="E14" s="0" t="inlineStr">
+          <t xml:space="preserve">Classification; Regression; Anomaly Detection; Subset Selection; Data Summarization</t>
+        </is>
+      </c>
+      <c r="E14" s="0">
+        <v>5</v>
+      </c>
+      <c r="F14" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="G14" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A30US3Ge</t>
         </is>
       </c>
-      <c r="F14" s="0" t="inlineStr">
+      <c r="H14" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A30</t>
         </is>
       </c>
-      <c r="G14" s="0" t="inlineStr">
+      <c r="I14" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Recidivism prediction with Decision Trees (criminal justice)</t>
         </is>
       </c>
-      <c r="H14" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Gemini_1.5_flash</t>
-        </is>
-      </c>
-      <c r="I14" s="0" t="inlineStr">
+      <c r="J14" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gemini_1.5_flash</t>
+        </is>
+      </c>
+      <c r="K14" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">judge or magistrate</t>
         </is>
       </c>
-      <c r="J14" s="0" t="inlineStr">
+      <c r="L14" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">As a judge or magistrate, I want to have access to objective and reliable information about a defendant's risk of re-offending to inform sentencing decisions.</t>
         </is>
@@ -795,35 +911,43 @@
       </c>
       <c r="D15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">High</t>
-        </is>
-      </c>
-      <c r="E15" s="0" t="inlineStr">
+          <t xml:space="preserve">Ranking; Matching; Pricing; Advertising; Entity Resolution; Sentiment Analysis; Bias Detection in Language Models</t>
+        </is>
+      </c>
+      <c r="E15" s="0">
+        <v>7</v>
+      </c>
+      <c r="F15" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="G15" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A24US6Ge</t>
         </is>
       </c>
-      <c r="F15" s="0" t="inlineStr">
+      <c r="H15" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A24</t>
         </is>
       </c>
-      <c r="G15" s="0" t="inlineStr">
+      <c r="I15" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">ArnetMiner academic search / academic social network</t>
         </is>
       </c>
-      <c r="H15" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Gemini_1.5_flash</t>
-        </is>
-      </c>
-      <c r="I15" s="0" t="inlineStr">
+      <c r="J15" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gemini_1.5_flash</t>
+        </is>
+      </c>
+      <c r="K15" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">research funder</t>
         </is>
       </c>
-      <c r="J15" s="0" t="inlineStr">
+      <c r="L15" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">As a research funder, I want to identify promising research areas and researchers for potential funding opportunities.</t>
         </is>
@@ -845,35 +969,43 @@
       </c>
       <c r="D16" s="0" t="inlineStr">
         <is>
+          <t xml:space="preserve">Classification; Regression; Ranking; Matching; Risk Assessment; Representation Learning; Anomaly Detection; Task Assignment; Spatio-Temporal Process Learning; Graph Diffusion; Graph Augmentation; Entity Resolution; Sentiment Analysis; Bias Detection in Word Embeddings; Bias Detection in Language Models; Machine Translation; Speech Recognition</t>
+        </is>
+      </c>
+      <c r="E16" s="0">
+        <v>17</v>
+      </c>
+      <c r="F16" s="0" t="inlineStr">
+        <is>
           <t xml:space="preserve">Medium</t>
         </is>
       </c>
-      <c r="E16" s="0" t="inlineStr">
+      <c r="G16" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A32US5Ge</t>
         </is>
       </c>
-      <c r="F16" s="0" t="inlineStr">
+      <c r="H16" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A32</t>
         </is>
       </c>
-      <c r="G16" s="0" t="inlineStr">
+      <c r="I16" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Stance detection with multi-task learning (NLP)</t>
         </is>
       </c>
-      <c r="H16" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Gemini_1.5_flash</t>
-        </is>
-      </c>
-      <c r="I16" s="0" t="inlineStr">
+      <c r="J16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gemini_1.5_flash</t>
+        </is>
+      </c>
+      <c r="K16" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">social media moderator</t>
         </is>
       </c>
-      <c r="J16" s="0" t="inlineStr">
+      <c r="L16" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">As a social media moderator, I want to prioritize content for review based on the intensity of a user's stance (e.g., strongly against vs. mildly disagreeing).</t>
         </is>
@@ -895,35 +1027,43 @@
       </c>
       <c r="D17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">High</t>
-        </is>
-      </c>
-      <c r="E17" s="0" t="inlineStr">
+          <t xml:space="preserve">Classification; Regression; Representation Learning; Clustering; Anomaly Detection; Spatio-Temporal Process Learning; Graph Diffusion; Graph Augmentation; Subset Selection; Data Summarization; Graph Mining; Sentiment Analysis; Bias Detection in Word Embeddings; Bias Detection in Language Models; Machine Translation; Speech Recognition</t>
+        </is>
+      </c>
+      <c r="E17" s="0">
+        <v>16</v>
+      </c>
+      <c r="F17" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="G17" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A17US1Ge</t>
         </is>
       </c>
-      <c r="F17" s="0" t="inlineStr">
+      <c r="H17" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A17</t>
         </is>
       </c>
-      <c r="G17" s="0" t="inlineStr">
+      <c r="I17" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Sleep apnea / hypopnea prediction with LAMSTAR neural networks</t>
         </is>
       </c>
-      <c r="H17" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Gemini_1.5_flash</t>
-        </is>
-      </c>
-      <c r="I17" s="0" t="inlineStr">
+      <c r="J17" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gemini_1.5_flash</t>
+        </is>
+      </c>
+      <c r="K17" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">sleep specialist</t>
         </is>
       </c>
-      <c r="J17" s="0" t="inlineStr">
+      <c r="L17" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">As a sleep specialist, I want to use an advanced prediction system to forecast episodes of apnea and hypopnea, enabling me to tailor treatment plans more effectively for individual patients.</t>
         </is>
@@ -945,35 +1085,43 @@
       </c>
       <c r="D18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">High</t>
-        </is>
-      </c>
-      <c r="E18" s="0" t="inlineStr">
+          <t xml:space="preserve">Classification</t>
+        </is>
+      </c>
+      <c r="E18" s="0">
+        <v>1</v>
+      </c>
+      <c r="F18" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="G18" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A39US1Ge</t>
         </is>
       </c>
-      <c r="F18" s="0" t="inlineStr">
+      <c r="H18" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A39</t>
         </is>
       </c>
-      <c r="G18" s="0" t="inlineStr">
+      <c r="I18" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Playlist success prediction</t>
         </is>
       </c>
-      <c r="H18" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Gemini_1.5_flash</t>
-        </is>
-      </c>
-      <c r="I18" s="0" t="inlineStr">
+      <c r="J18" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gemini_1.5_flash</t>
+        </is>
+      </c>
+      <c r="K18" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">music enthusiast</t>
         </is>
       </c>
-      <c r="J18" s="0" t="inlineStr">
+      <c r="L18" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">As a music enthusiast, I want to create playlists that resonate with a wider audience and gain popularity. I want a tool that can predict the success of my playlists based on musical characteristics, allowing me to refine my curation and increase engagement.</t>
         </is>
@@ -995,35 +1143,43 @@
       </c>
       <c r="D19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">High</t>
-        </is>
-      </c>
-      <c r="E19" s="0" t="inlineStr">
+          <t xml:space="preserve">Ranking; Matching; Pricing; Advertising; Entity Resolution; Sentiment Analysis; Bias Detection in Language Models</t>
+        </is>
+      </c>
+      <c r="E19" s="0">
+        <v>7</v>
+      </c>
+      <c r="F19" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="G19" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A33US2Ll</t>
         </is>
       </c>
-      <c r="F19" s="0" t="inlineStr">
+      <c r="H19" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A33</t>
         </is>
       </c>
-      <c r="G19" s="0" t="inlineStr">
+      <c r="I19" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Semantic news search with Wikidata annotation</t>
         </is>
       </c>
-      <c r="H19" s="0" t="inlineStr">
+      <c r="J19" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Llama 3.1 70b</t>
         </is>
       </c>
-      <c r="I19" s="0" t="inlineStr">
+      <c r="K19" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">news agency</t>
         </is>
       </c>
-      <c r="J19" s="0" t="inlineStr">
+      <c r="L19" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">As a news agency, I want to be able to search for precise facts described in news articles, so that I can verify information and ensure the accuracy of our reporting.</t>
         </is>
@@ -1045,35 +1201,43 @@
       </c>
       <c r="D20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">High</t>
-        </is>
-      </c>
-      <c r="E20" s="0" t="inlineStr">
+          <t xml:space="preserve">Classification</t>
+        </is>
+      </c>
+      <c r="E20" s="0">
+        <v>1</v>
+      </c>
+      <c r="F20" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="G20" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A16US1Ge</t>
         </is>
       </c>
-      <c r="F20" s="0" t="inlineStr">
+      <c r="H20" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A16</t>
         </is>
       </c>
-      <c r="G20" s="0" t="inlineStr">
+      <c r="I20" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Newborn cry diagnostic system (cry-audio classification)</t>
         </is>
       </c>
-      <c r="H20" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Gemini_1.5_flash</t>
-        </is>
-      </c>
-      <c r="I20" s="0" t="inlineStr">
+      <c r="J20" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gemini_1.5_flash</t>
+        </is>
+      </c>
+      <c r="K20" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">pediatrician</t>
         </is>
       </c>
-      <c r="J20" s="0" t="inlineStr">
+      <c r="L20" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">As a pediatrician, I want a non-invasive tool that can analyze a newborn's cry and help me identify potential health issues early on.</t>
         </is>
@@ -1095,35 +1259,43 @@
       </c>
       <c r="D21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">High</t>
-        </is>
-      </c>
-      <c r="E21" s="0" t="inlineStr">
+          <t xml:space="preserve">Classification; Regression; Ranking; Matching; Risk Assessment; Representation Learning; Clustering; Anomaly Detection; Districting; Task Assignment; Spatio-Temporal Process Learning; Graph Diffusion; Graph Augmentation; Resource Allocation; Subset Selection; Data Summarization; Graph Mining; Pricing; Advertising; Entity Resolution; Sentiment Analysis; Bias Detection in Word Embeddings; Bias Detection in Language Models; Machine Translation; Speech Recognition</t>
+        </is>
+      </c>
+      <c r="E21" s="0">
+        <v>25</v>
+      </c>
+      <c r="F21" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="G21" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A13US2Ge</t>
         </is>
       </c>
-      <c r="F21" s="0" t="inlineStr">
+      <c r="H21" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A13</t>
         </is>
       </c>
-      <c r="G21" s="0" t="inlineStr">
+      <c r="I21" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">AI-DrugNet drug repurposing for Alzheimer’s disease</t>
         </is>
       </c>
-      <c r="H21" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Gemini_1.5_flash</t>
-        </is>
-      </c>
-      <c r="I21" s="0" t="inlineStr">
+      <c r="J21" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gemini_1.5_flash</t>
+        </is>
+      </c>
+      <c r="K21" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">pharmaceutical company scientist</t>
         </is>
       </c>
-      <c r="J21" s="0" t="inlineStr">
+      <c r="L21" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">As a pharmaceutical company scientist, I want the platform to predict potential combinations of existing drugs that may have a synergistic effect in treating AD.</t>
         </is>
@@ -1145,35 +1317,43 @@
       </c>
       <c r="D22" s="0" t="inlineStr">
         <is>
+          <t xml:space="preserve">Districting; Task Assignment; Resource Allocation; Pricing; Advertising</t>
+        </is>
+      </c>
+      <c r="E22" s="0">
+        <v>5</v>
+      </c>
+      <c r="F22" s="0" t="inlineStr">
+        <is>
           <t xml:space="preserve">Low</t>
         </is>
       </c>
-      <c r="E22" s="0" t="inlineStr">
+      <c r="G22" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A4US1Ge</t>
         </is>
       </c>
-      <c r="F22" s="0" t="inlineStr">
+      <c r="H22" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A4</t>
         </is>
       </c>
-      <c r="G22" s="0" t="inlineStr">
+      <c r="I22" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">AI-powered military drones &amp; international security</t>
         </is>
       </c>
-      <c r="H22" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Gemini_1.5_flash</t>
-        </is>
-      </c>
-      <c r="I22" s="0" t="inlineStr">
+      <c r="J22" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gemini_1.5_flash</t>
+        </is>
+      </c>
+      <c r="K22" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">military commander</t>
         </is>
       </c>
-      <c r="J22" s="0" t="inlineStr">
+      <c r="L22" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">As a military leader, I want to leverage AI for improved situational awareness and faster decision- making on the battlefield to gain a tactical advantage.</t>
         </is>
@@ -1195,35 +1375,43 @@
       </c>
       <c r="D23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">High</t>
-        </is>
-      </c>
-      <c r="E23" s="0" t="inlineStr">
+          <t xml:space="preserve">Classification; Representation Learning; Clustering; Anomaly Detection; Data Summarization; Graph Mining; Entity Resolution</t>
+        </is>
+      </c>
+      <c r="E23" s="0">
+        <v>7</v>
+      </c>
+      <c r="F23" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="G23" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A18US1Ge</t>
         </is>
       </c>
-      <c r="F23" s="0" t="inlineStr">
+      <c r="H23" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A18</t>
         </is>
       </c>
-      <c r="G23" s="0" t="inlineStr">
+      <c r="I23" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Tuberculosis detection from chest X-rays with CNNs</t>
         </is>
       </c>
-      <c r="H23" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Gemini_1.5_flash</t>
-        </is>
-      </c>
-      <c r="I23" s="0" t="inlineStr">
+      <c r="J23" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gemini_1.5_flash</t>
+        </is>
+      </c>
+      <c r="K23" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">radiologist</t>
         </is>
       </c>
-      <c r="J23" s="0" t="inlineStr">
+      <c r="L23" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">As a radiologist, I want a tool that can assist me in diagnosing TB disease from chest X-rays, improving accuracy and efficiency in my workflow.</t>
         </is>
@@ -1245,35 +1433,43 @@
       </c>
       <c r="D24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">High</t>
-        </is>
-      </c>
-      <c r="E24" s="0" t="inlineStr">
+          <t xml:space="preserve">Sentiment Analysis; Bias Detection in Language Models; Machine Translation; Speech Recognition</t>
+        </is>
+      </c>
+      <c r="E24" s="0">
+        <v>4</v>
+      </c>
+      <c r="F24" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="G24" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A3US2Ge</t>
         </is>
       </c>
-      <c r="F24" s="0" t="inlineStr">
+      <c r="H24" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A3</t>
         </is>
       </c>
-      <c r="G24" s="0" t="inlineStr">
+      <c r="I24" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Real-time aggression detection on Twitter</t>
         </is>
       </c>
-      <c r="H24" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Gemini_1.5_flash</t>
-        </is>
-      </c>
-      <c r="I24" s="0" t="inlineStr">
+      <c r="J24" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gemini_1.5_flash</t>
+        </is>
+      </c>
+      <c r="K24" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">moderator</t>
         </is>
       </c>
-      <c r="J24" s="0" t="inlineStr">
+      <c r="L24" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">As a content moderator, I want a tool that identifies potentially aggressive tweets with high accuracy so that I can prioritize them for review and take appropriate action.</t>
         </is>
@@ -1295,35 +1491,43 @@
       </c>
       <c r="D25" s="0" t="inlineStr">
         <is>
+          <t xml:space="preserve">Classification; Regression; Ranking; Representation Learning; Clustering; Anomaly Detection; Districting; Graph Mining; Pricing; Advertising; Entity Resolution; Sentiment Analysis; Bias Detection in Word Embeddings; Bias Detection in Language Models</t>
+        </is>
+      </c>
+      <c r="E25" s="0">
+        <v>14</v>
+      </c>
+      <c r="F25" s="0" t="inlineStr">
+        <is>
           <t xml:space="preserve">Low</t>
         </is>
       </c>
-      <c r="E25" s="0" t="inlineStr">
+      <c r="G25" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A12US7O1</t>
         </is>
       </c>
-      <c r="F25" s="0" t="inlineStr">
+      <c r="H25" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A12</t>
         </is>
       </c>
-      <c r="G25" s="0" t="inlineStr">
+      <c r="I25" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Firearm Violence Vulnerability Index (XGBoost community-risk forecasting)</t>
         </is>
       </c>
-      <c r="H25" s="0" t="inlineStr">
+      <c r="J25" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">O1_mini</t>
         </is>
       </c>
-      <c r="I25" s="0" t="inlineStr">
+      <c r="K25" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">grant writer</t>
         </is>
       </c>
-      <c r="J25" s="0" t="inlineStr">
+      <c r="L25" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">As a grant writer, I want to utilize the FVVI’s standardized risk assessments, so that I can secure funding for targeted violence prevention programs.</t>
         </is>
@@ -1345,41 +1549,49 @@
       </c>
       <c r="D26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">High</t>
-        </is>
-      </c>
-      <c r="E26" s="0" t="inlineStr">
+          <t xml:space="preserve">Classification; Regression; Clustering; Anomaly Detection; Data Summarization; Graph Mining; Entity Resolution</t>
+        </is>
+      </c>
+      <c r="E26" s="0">
+        <v>7</v>
+      </c>
+      <c r="F26" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="G26" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A37US1Ge</t>
         </is>
       </c>
-      <c r="F26" s="0" t="inlineStr">
+      <c r="H26" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A37</t>
         </is>
       </c>
-      <c r="G26" s="0" t="inlineStr">
+      <c r="I26" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Fantasy sports analytics &amp; player selection</t>
         </is>
       </c>
-      <c r="H26" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Gemini_1.5_flash</t>
-        </is>
-      </c>
-      <c r="I26" s="0" t="inlineStr">
+      <c r="J26" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gemini_1.5_flash</t>
+        </is>
+      </c>
+      <c r="K26" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">sports fan</t>
         </is>
       </c>
-      <c r="J26" s="0" t="inlineStr">
+      <c r="L26" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">As a casual sports fan, I want to participate in fantasy sports but feel overwhelmed by the amount of information and player choices. I want a platform that uses data and analytics to help me make informed decisions about which players to select for my team.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J26"/>
+  <autoFilter ref="A1:L26"/>
 </worksheet>
 </file>
</xml_diff>